<commit_message>
cgg animal plant upload works
</commit_message>
<xml_diff>
--- a/static/example_sheets/CGG Sediment Water.xlsx
+++ b/static/example_sheets/CGG Sediment Water.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\glj523\Documents\github repoes\upload_web_app\static\example_sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\magnu\Documents\Git Repoes\gg-metadatabase-ui\static\example_sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B6DFCC-590C-4712-BCFB-37910E4467E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00254931-6BD8-45C2-9FCB-EFCD7BF10F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{F20BE04D-14A6-4DFA-9322-DA461E992517}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F20BE04D-14A6-4DFA-9322-DA461E992517}"/>
   </bookViews>
   <sheets>
     <sheet name="eDNA_Archive_sampling_(20231027" sheetId="2" r:id="rId1"/>
@@ -1038,7 +1038,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="108">
   <si>
     <t>Expected column names and positions:</t>
   </si>
@@ -1359,6 +1359,9 @@
   </si>
   <si>
     <t>[10, 50)</t>
+  </si>
+  <si>
+    <t>2024-31-01</t>
   </si>
 </sst>
 </file>
@@ -1502,14 +1505,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1534,6 +1535,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma 2" xfId="3" xr:uid="{8942F21F-F0D4-468F-A2D9-2DD07A9F09D0}"/>
@@ -1818,9 +1820,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022 Tema">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1858,7 +1860,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1964,7 +1966,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2106,7 +2108,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2168,7 +2170,7 @@
     <col min="51" max="51" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" s="5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:50" s="3" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2320,445 +2322,445 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:50" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="1">
-        <v>45321</v>
-      </c>
-      <c r="I2" s="1">
-        <v>45321</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="2">
         <v>10</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="R2">
+      <c r="R2" s="2">
         <v>10</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="T2" t="s">
+      <c r="T2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="U2" t="s">
+      <c r="U2" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="V2" t="s">
+      <c r="V2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="X2" t="s">
+      <c r="X2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Y2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="Z2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AA2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AB2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AC2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AD2" s="4">
+      <c r="AD2" s="11">
         <v>61.139899999999997</v>
       </c>
-      <c r="AE2">
+      <c r="AE2" s="2">
         <v>-45.534700000000001</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AF2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AG2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AH2" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AI2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AJ2" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AK2" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AL2" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AM2" t="s">
+      <c r="AJ2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AK2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AL2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AM2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AP2" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AW2" t="s">
+      <c r="AP2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AW2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="AX2" t="b">
+      <c r="AX2" s="2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
+    <row r="3" spans="1:50" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G3" s="1">
-        <v>45321</v>
-      </c>
-      <c r="I3" s="1">
-        <v>45321</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="G3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="2">
         <v>200</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="R3">
+      <c r="R3" s="2">
         <v>10</v>
       </c>
-      <c r="S3" t="s">
+      <c r="S3" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="T3" t="s">
+      <c r="T3" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="U3" t="s">
+      <c r="U3" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="V3" t="s">
+      <c r="V3" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="W3" t="s">
+      <c r="W3" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="X3" t="s">
+      <c r="X3" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Y3" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="Z3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AA3" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="AB3" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AC3" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AD3" s="4">
+      <c r="AD3" s="11">
         <v>61.139899999999997</v>
       </c>
-      <c r="AE3">
+      <c r="AE3" s="2">
         <v>-45.534700000000001</v>
       </c>
-      <c r="AF3" t="s">
+      <c r="AF3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AG3" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AH3" t="s">
+      <c r="AH3" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AI3" t="s">
+      <c r="AI3" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AJ3" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AK3" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AL3" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AM3" t="s">
+      <c r="AJ3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AK3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AL3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AM3" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AP3" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AW3" t="s">
+      <c r="AP3" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AW3" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="AX3" t="b">
+      <c r="AX3" s="2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
+    <row r="4" spans="1:50" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G4" s="1">
-        <v>45321</v>
-      </c>
-      <c r="I4" s="1">
-        <v>45321</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="G4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="2">
         <v>300.3</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q4" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="R4">
+      <c r="R4" s="2">
         <v>10.5</v>
       </c>
-      <c r="S4" t="s">
+      <c r="S4" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="T4" t="s">
+      <c r="T4" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="U4" t="s">
+      <c r="U4" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="V4" t="s">
+      <c r="V4" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="W4" t="s">
+      <c r="W4" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="X4" t="s">
+      <c r="X4" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Y4" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="Z4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AA4" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="AB4" t="s">
+      <c r="AB4" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AC4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="AD4" s="4">
+      <c r="AD4" s="11">
         <v>61.139899999999997</v>
       </c>
-      <c r="AE4">
+      <c r="AE4" s="2">
         <v>-45.534700000000001</v>
       </c>
-      <c r="AF4" t="s">
+      <c r="AF4" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="AG4" t="s">
+      <c r="AG4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AH4" t="s">
+      <c r="AH4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="AI4" t="s">
+      <c r="AI4" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="AJ4" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AK4" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AL4" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AM4" t="s">
+      <c r="AJ4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AK4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AL4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AM4" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AP4" s="1">
-        <v>45321</v>
-      </c>
-      <c r="AW4" t="s">
+      <c r="AP4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="AW4" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="AX4" t="b">
+      <c r="AX4" s="2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:50" s="6" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:50" s="4" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="M5" s="6" t="s">
+      <c r="M5" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="N5" s="6" t="s">
+      <c r="N5" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="R5" s="6" t="s">
+      <c r="R5" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="U5" s="6" t="s">
+      <c r="U5" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="AD5" s="7" t="s">
+      <c r="AD5" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="AE5" s="7" t="s">
+      <c r="AE5" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="AG5" s="6" t="s">
+      <c r="AG5" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="AJ5" s="6" t="s">
+      <c r="AJ5" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="AK5" s="6" t="s">
+      <c r="AK5" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="AL5" s="6" t="s">
+      <c r="AL5" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="AP5" s="6" t="s">
+      <c r="AP5" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:50" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+    <row r="6" spans="1:50" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="AD6" s="9"/>
+      <c r="AD6" s="7"/>
     </row>
-    <row r="7" spans="1:50" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
+    <row r="7" spans="1:50" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="N7" s="8" t="s">
+      <c r="N7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="O7" s="10"/>
-      <c r="AB7" s="8" t="s">
+      <c r="O7" s="8"/>
+      <c r="AB7" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="AD7" s="9" t="s">
+      <c r="AD7" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="AE7" s="8" t="s">
+      <c r="AE7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="AG7" s="8" t="s">
+      <c r="AG7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="AJ7" s="8" t="s">
+      <c r="AJ7" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:50" s="6" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+    <row r="8" spans="1:50" s="4" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="L8" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="M8" s="6" t="s">
+      <c r="M8" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="N8" s="6" t="s">
+      <c r="N8" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="S8" s="6" t="s">
+      <c r="S8" s="4" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2783,9 +2785,10 @@
     <hyperlink ref="AI2" r:id="rId1" xr:uid="{B2B44199-098D-43B8-88D1-A75F443FF608}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>